<commit_message>
fix template for pictures location
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/cards/ZAccreditation.xlsx
+++ b/owlcms/src/main/resources/templates/cards/ZAccreditation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\cards\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033A5B13-929F-4F08-9093-169130D6129C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109AC222-4DCA-4196-8736-481915E15955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>jx:image(src="local.getBytes('_pictures/'+a.membership+'.jpg')" imageType="JPEG" lastCell="A2")</t>
+          <t>jx:image(src="local.getBytes('pictures/'+a.membership+'.jpg')" imageType="JPEG" lastCell="A2")</t>
         </r>
         <r>
           <rPr>

</xml_diff>

<commit_message>
accreditation template + instructions
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/cards/ZAccreditation.xlsx
+++ b/owlcms/src/main/resources/templates/cards/ZAccreditation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15E4F4B-F2AC-4B09-93A9-8607E389F896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5853BDE2-40A7-4676-A5FE-C6C2FB41E80B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -127,10 +127,10 @@
     <t>Live Feed QR Code</t>
   </si>
   <si>
-    <t>${athlete.group}</t>
+    <t>sponsor logos</t>
   </si>
   <si>
-    <t>sponsor logos</t>
+    <t>${t.get("Group")} ${athlete.group} - ${athlete.group.localizedStartDay} ${athlete.group.localizedStartHour}</t>
   </si>
 </sst>
 </file>
@@ -896,7 +896,7 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="1" max="1" width="0.85546875" customWidth="1"/>
     <col min="2" max="2" width="2.42578125" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
     <col min="4" max="4" width="3.5703125" customWidth="1"/>
@@ -949,7 +949,7 @@
     <row r="5" spans="1:9" s="14" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B5" s="15"/>
       <c r="C5" s="34" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="34"/>
       <c r="E5" s="34"/>
@@ -1028,7 +1028,7 @@
     <row r="14" spans="1:9" s="21" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="22"/>
       <c r="C14" s="32" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="32"/>
       <c r="E14" s="32"/>
@@ -1111,8 +1111,8 @@
     <mergeCell ref="E10:G12"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.01" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0" right="0.39370078740157483" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" r:id="rId1"/>
   <headerFooter scaleWithDoc="0"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>